<commit_message>
Fix import preview filtering
</commit_message>
<xml_diff>
--- a/public/templates/otzar_hakodesh_books_import_template.xlsx
+++ b/public/templates/otzar_hakodesh_books_import_template.xlsx
@@ -804,7 +804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1033,100 +1033,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>7290000000011</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>חומשים לדוגמה</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>תת קטגוריה לדוגמה</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>ספרי יסוד|מומלצים</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>מחבר לדוגמה</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>רב לדוגמה</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>הוצאה לדוגמה</t>
-        </is>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>תיאור קצר שיופיע בכרטיס המוצר</t>
-        </is>
-      </c>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
-          <t>תיאור מפורט שיופיע בדף המוצר</t>
-        </is>
-      </c>
-      <c r="K3" s="8" t="n">
-        <v>120</v>
-      </c>
-      <c r="L3" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="M3" s="8" t="n">
-        <v>25</v>
-      </c>
-      <c r="N3" s="8" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="O3" s="8" t="inlineStr">
-        <is>
-          <t>עברית</t>
-        </is>
-      </c>
-      <c r="P3" s="8" t="inlineStr">
-        <is>
-          <t>001.jpg</t>
-        </is>
-      </c>
-      <c r="Q3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="R3" s="8" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="S3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="T3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-    </row>
+    <row r="3" ht="24" customHeight="1"/>
     <row r="4" ht="24" customHeight="1"/>
     <row r="5" ht="24" customHeight="1"/>
     <row r="6" ht="24" customHeight="1"/>
@@ -3145,7 +3052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3374,100 +3281,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>7290000000011</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>גמרות ומשניות לדוגמה</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>תת קטגוריה לדוגמה</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>ספרי יסוד|מומלצים</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>מחבר לדוגמה</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>רב לדוגמה</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>הוצאה לדוגמה</t>
-        </is>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>תיאור קצר שיופיע בכרטיס המוצר</t>
-        </is>
-      </c>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
-          <t>תיאור מפורט שיופיע בדף המוצר</t>
-        </is>
-      </c>
-      <c r="K3" s="8" t="n">
-        <v>120</v>
-      </c>
-      <c r="L3" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="M3" s="8" t="n">
-        <v>25</v>
-      </c>
-      <c r="N3" s="8" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="O3" s="8" t="inlineStr">
-        <is>
-          <t>עברית</t>
-        </is>
-      </c>
-      <c r="P3" s="8" t="inlineStr">
-        <is>
-          <t>001.jpg</t>
-        </is>
-      </c>
-      <c r="Q3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="R3" s="8" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="S3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="T3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-    </row>
+    <row r="3" ht="24" customHeight="1"/>
     <row r="4" ht="24" customHeight="1"/>
     <row r="5" ht="24" customHeight="1"/>
     <row r="6" ht="24" customHeight="1"/>
@@ -5486,7 +5300,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5715,100 +5529,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>7290000000011</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>הלכה לדוגמה</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>תת קטגוריה לדוגמה</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>ספרי יסוד|מומלצים</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>מחבר לדוגמה</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>רב לדוגמה</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>הוצאה לדוגמה</t>
-        </is>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>תיאור קצר שיופיע בכרטיס המוצר</t>
-        </is>
-      </c>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
-          <t>תיאור מפורט שיופיע בדף המוצר</t>
-        </is>
-      </c>
-      <c r="K3" s="8" t="n">
-        <v>120</v>
-      </c>
-      <c r="L3" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="M3" s="8" t="n">
-        <v>25</v>
-      </c>
-      <c r="N3" s="8" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="O3" s="8" t="inlineStr">
-        <is>
-          <t>עברית</t>
-        </is>
-      </c>
-      <c r="P3" s="8" t="inlineStr">
-        <is>
-          <t>001.jpg</t>
-        </is>
-      </c>
-      <c r="Q3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="R3" s="8" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="S3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="T3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-    </row>
+    <row r="3" ht="24" customHeight="1"/>
     <row r="4" ht="24" customHeight="1"/>
     <row r="5" ht="24" customHeight="1"/>
     <row r="6" ht="24" customHeight="1"/>
@@ -7827,7 +7548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -8056,100 +7777,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>7290000000011</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>חסידות וקבלה לדוגמה</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>תת קטגוריה לדוגמה</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>ספרי יסוד|מומלצים</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>מחבר לדוגמה</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>רב לדוגמה</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>הוצאה לדוגמה</t>
-        </is>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>תיאור קצר שיופיע בכרטיס המוצר</t>
-        </is>
-      </c>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
-          <t>תיאור מפורט שיופיע בדף המוצר</t>
-        </is>
-      </c>
-      <c r="K3" s="8" t="n">
-        <v>120</v>
-      </c>
-      <c r="L3" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="M3" s="8" t="n">
-        <v>25</v>
-      </c>
-      <c r="N3" s="8" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="O3" s="8" t="inlineStr">
-        <is>
-          <t>עברית</t>
-        </is>
-      </c>
-      <c r="P3" s="8" t="inlineStr">
-        <is>
-          <t>001.jpg</t>
-        </is>
-      </c>
-      <c r="Q3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="R3" s="8" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="S3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="T3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-    </row>
+    <row r="3" ht="24" customHeight="1"/>
     <row r="4" ht="24" customHeight="1"/>
     <row r="5" ht="24" customHeight="1"/>
     <row r="6" ht="24" customHeight="1"/>
@@ -10168,7 +9796,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -10397,100 +10025,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>7290000000011</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>ספרי ילדים ונוער לדוגמה</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>תת קטגוריה לדוגמה</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>ספרי יסוד|מומלצים</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>מחבר לדוגמה</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>רב לדוגמה</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>הוצאה לדוגמה</t>
-        </is>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>תיאור קצר שיופיע בכרטיס המוצר</t>
-        </is>
-      </c>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
-          <t>תיאור מפורט שיופיע בדף המוצר</t>
-        </is>
-      </c>
-      <c r="K3" s="8" t="n">
-        <v>120</v>
-      </c>
-      <c r="L3" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="M3" s="8" t="n">
-        <v>25</v>
-      </c>
-      <c r="N3" s="8" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="O3" s="8" t="inlineStr">
-        <is>
-          <t>עברית</t>
-        </is>
-      </c>
-      <c r="P3" s="8" t="inlineStr">
-        <is>
-          <t>001.jpg</t>
-        </is>
-      </c>
-      <c r="Q3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="R3" s="8" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="S3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="T3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-    </row>
+    <row r="3" ht="24" customHeight="1"/>
     <row r="4" ht="24" customHeight="1"/>
     <row r="5" ht="24" customHeight="1"/>
     <row r="6" ht="24" customHeight="1"/>
@@ -12509,7 +12044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -12738,100 +12273,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>7290000000011</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>מוסר ומחשבה לדוגמה</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>תת קטגוריה לדוגמה</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>ספרי יסוד|מומלצים</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>מחבר לדוגמה</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>רב לדוגמה</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>הוצאה לדוגמה</t>
-        </is>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>תיאור קצר שיופיע בכרטיס המוצר</t>
-        </is>
-      </c>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
-          <t>תיאור מפורט שיופיע בדף המוצר</t>
-        </is>
-      </c>
-      <c r="K3" s="8" t="n">
-        <v>120</v>
-      </c>
-      <c r="L3" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="M3" s="8" t="n">
-        <v>25</v>
-      </c>
-      <c r="N3" s="8" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="O3" s="8" t="inlineStr">
-        <is>
-          <t>עברית</t>
-        </is>
-      </c>
-      <c r="P3" s="8" t="inlineStr">
-        <is>
-          <t>001.jpg</t>
-        </is>
-      </c>
-      <c r="Q3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="R3" s="8" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="S3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="T3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-    </row>
+    <row r="3" ht="24" customHeight="1"/>
     <row r="4" ht="24" customHeight="1"/>
     <row r="5" ht="24" customHeight="1"/>
     <row r="6" ht="24" customHeight="1"/>
@@ -14850,7 +14292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -15079,100 +14521,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>7290000000011</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>ספרי הרב עובדיה יוסף לדוגמה</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>תת קטגוריה לדוגמה</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>ספרי יסוד|מומלצים</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>מחבר לדוגמה</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>רב לדוגמה</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>הוצאה לדוגמה</t>
-        </is>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>תיאור קצר שיופיע בכרטיס המוצר</t>
-        </is>
-      </c>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
-          <t>תיאור מפורט שיופיע בדף המוצר</t>
-        </is>
-      </c>
-      <c r="K3" s="8" t="n">
-        <v>120</v>
-      </c>
-      <c r="L3" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="M3" s="8" t="n">
-        <v>25</v>
-      </c>
-      <c r="N3" s="8" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="O3" s="8" t="inlineStr">
-        <is>
-          <t>עברית</t>
-        </is>
-      </c>
-      <c r="P3" s="8" t="inlineStr">
-        <is>
-          <t>001.jpg</t>
-        </is>
-      </c>
-      <c r="Q3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="R3" s="8" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="S3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="T3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-    </row>
+    <row r="3" ht="24" customHeight="1"/>
     <row r="4" ht="24" customHeight="1"/>
     <row r="5" ht="24" customHeight="1"/>
     <row r="6" ht="24" customHeight="1"/>
@@ -17191,7 +16540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -17420,100 +16769,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>7290000000011</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>ספרי חב"ד לדוגמה</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>תת קטגוריה לדוגמה</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>ספרי יסוד|מומלצים</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>מחבר לדוגמה</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>רב לדוגמה</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>הוצאה לדוגמה</t>
-        </is>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>תיאור קצר שיופיע בכרטיס המוצר</t>
-        </is>
-      </c>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
-          <t>תיאור מפורט שיופיע בדף המוצר</t>
-        </is>
-      </c>
-      <c r="K3" s="8" t="n">
-        <v>120</v>
-      </c>
-      <c r="L3" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="M3" s="8" t="n">
-        <v>25</v>
-      </c>
-      <c r="N3" s="8" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="O3" s="8" t="inlineStr">
-        <is>
-          <t>עברית</t>
-        </is>
-      </c>
-      <c r="P3" s="8" t="inlineStr">
-        <is>
-          <t>001.jpg</t>
-        </is>
-      </c>
-      <c r="Q3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="R3" s="8" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="S3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="T3" s="8" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-    </row>
+    <row r="3" ht="24" customHeight="1"/>
     <row r="4" ht="24" customHeight="1"/>
     <row r="5" ht="24" customHeight="1"/>
     <row r="6" ht="24" customHeight="1"/>

</xml_diff>

<commit_message>
Treat import numbers as local
</commit_message>
<xml_diff>
--- a/public/templates/otzar_hakodesh_books_import_template.xlsx
+++ b/public/templates/otzar_hakodesh_books_import_template.xlsx
@@ -459,7 +459,7 @@
   <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
@@ -468,13 +468,13 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>מק"ט</t>
+          <t>מספר</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
@@ -519,7 +519,7 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>תמונה</t>
+          <t>מספר תמונה</t>
         </is>
       </c>
     </row>
@@ -539,7 +539,7 @@
   <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
@@ -548,13 +548,13 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>מק"ט</t>
+          <t>מספר</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
@@ -599,7 +599,7 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>תמונה</t>
+          <t>מספר תמונה</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
   <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
@@ -628,13 +628,13 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>מק"ט</t>
+          <t>מספר</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>תמונה</t>
+          <t>מספר תמונה</t>
         </is>
       </c>
     </row>
@@ -699,7 +699,7 @@
   <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
@@ -708,13 +708,13 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>מק"ט</t>
+          <t>מספר</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>תמונה</t>
+          <t>מספר תמונה</t>
         </is>
       </c>
     </row>
@@ -779,7 +779,7 @@
   <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
@@ -788,13 +788,13 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>מק"ט</t>
+          <t>מספר</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
@@ -839,7 +839,7 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>תמונה</t>
+          <t>מספר תמונה</t>
         </is>
       </c>
     </row>
@@ -859,7 +859,7 @@
   <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
@@ -868,13 +868,13 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>מק"ט</t>
+          <t>מספר</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
@@ -919,7 +919,7 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>תמונה</t>
+          <t>מספר תמונה</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
   <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
@@ -948,13 +948,13 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>מק"ט</t>
+          <t>מספר</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
@@ -999,7 +999,7 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>תמונה</t>
+          <t>מספר תמונה</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
   <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
@@ -1028,13 +1028,13 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>מק"ט</t>
+          <t>מספר</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>תמונה</t>
+          <t>מספר תמונה</t>
         </is>
       </c>
     </row>

</xml_diff>